<commit_message>
Show viewability to 2 decimals in callouts
</commit_message>
<xml_diff>
--- a/output/2026-09/AS_Inventory_Report_2026-09.xlsx
+++ b/output/2026-09/AS_Inventory_Report_2026-09.xlsx
@@ -653,7 +653,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Custom in-game inventory, AdOps-approved scope (17 campaigns). Generated 2026-10-19 20:55. Synthetic portfolio data.</t>
+          <t>Custom in-game inventory, AdOps-approved scope (17 campaigns). Generated 2026-10-19 21:00. Synthetic portfolio data.</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
         <v>1220.6</v>
       </c>
       <c r="J22" s="14" t="n">
-        <v>14.96385926198357</v>
+        <v>14.96385926198356</v>
       </c>
       <c r="K22" s="15" t="n">
         <v>1.180957728402984</v>
@@ -1216,7 +1216,7 @@
         <v>1220.6</v>
       </c>
       <c r="M5" s="14" t="n">
-        <v>14.96385926198357</v>
+        <v>14.96385926198356</v>
       </c>
       <c r="N5" s="15" t="n">
         <v>1.180957728402984</v>

</xml_diff>